<commit_message>
Updated results with correct numbers (276 clean, 15 rejected, 92% quality score)
</commit_message>
<xml_diff>
--- a/output/error_log.xlsx
+++ b/output/error_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E678"/>
+  <dimension ref="A1:E674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16780,14 +16780,18 @@
     </row>
     <row r="668">
       <c r="A668" t="n">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="B668" t="inlineStr">
         <is>
           <t>Emp ID</t>
         </is>
       </c>
-      <c r="C668" t="inlineStr"/>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>EMP1264</t>
+        </is>
+      </c>
       <c r="D668" t="inlineStr">
         <is>
           <t>Duplicate employee ID</t>
@@ -16801,7 +16805,7 @@
     </row>
     <row r="669">
       <c r="A669" t="n">
-        <v>137</v>
+        <v>214</v>
       </c>
       <c r="B669" t="inlineStr">
         <is>
@@ -16810,7 +16814,7 @@
       </c>
       <c r="C669" t="inlineStr">
         <is>
-          <t>EMP1264</t>
+          <t>EMP1032</t>
         </is>
       </c>
       <c r="D669" t="inlineStr">
@@ -16826,14 +16830,18 @@
     </row>
     <row r="670">
       <c r="A670" t="n">
-        <v>184</v>
+        <v>232</v>
       </c>
       <c r="B670" t="inlineStr">
         <is>
           <t>Emp ID</t>
         </is>
       </c>
-      <c r="C670" t="inlineStr"/>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>EMP1288</t>
+        </is>
+      </c>
       <c r="D670" t="inlineStr">
         <is>
           <t>Duplicate employee ID</t>
@@ -16847,14 +16855,18 @@
     </row>
     <row r="671">
       <c r="A671" t="n">
-        <v>205</v>
+        <v>243</v>
       </c>
       <c r="B671" t="inlineStr">
         <is>
           <t>Emp ID</t>
         </is>
       </c>
-      <c r="C671" t="inlineStr"/>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>EMP1190</t>
+        </is>
+      </c>
       <c r="D671" t="inlineStr">
         <is>
           <t>Duplicate employee ID</t>
@@ -16868,7 +16880,7 @@
     </row>
     <row r="672">
       <c r="A672" t="n">
-        <v>214</v>
+        <v>246</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -16877,7 +16889,7 @@
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>EMP1032</t>
+          <t>EMP1266</t>
         </is>
       </c>
       <c r="D672" t="inlineStr">
@@ -16893,7 +16905,7 @@
     </row>
     <row r="673">
       <c r="A673" t="n">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="B673" t="inlineStr">
         <is>
@@ -16902,7 +16914,7 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>EMP1288</t>
+          <t>EMP1081</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
@@ -16918,7 +16930,7 @@
     </row>
     <row r="674">
       <c r="A674" t="n">
-        <v>243</v>
+        <v>285</v>
       </c>
       <c r="B674" t="inlineStr">
         <is>
@@ -16927,7 +16939,7 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>EMP1190</t>
+          <t>EMP1070</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
@@ -16936,102 +16948,6 @@
         </is>
       </c>
       <c r="E674" t="inlineStr">
-        <is>
-          <t>Row removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="675">
-      <c r="A675" t="n">
-        <v>246</v>
-      </c>
-      <c r="B675" t="inlineStr">
-        <is>
-          <t>Emp ID</t>
-        </is>
-      </c>
-      <c r="C675" t="inlineStr">
-        <is>
-          <t>EMP1266</t>
-        </is>
-      </c>
-      <c r="D675" t="inlineStr">
-        <is>
-          <t>Duplicate employee ID</t>
-        </is>
-      </c>
-      <c r="E675" t="inlineStr">
-        <is>
-          <t>Row removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="676">
-      <c r="A676" t="n">
-        <v>256</v>
-      </c>
-      <c r="B676" t="inlineStr">
-        <is>
-          <t>Emp ID</t>
-        </is>
-      </c>
-      <c r="C676" t="inlineStr">
-        <is>
-          <t>EMP1081</t>
-        </is>
-      </c>
-      <c r="D676" t="inlineStr">
-        <is>
-          <t>Duplicate employee ID</t>
-        </is>
-      </c>
-      <c r="E676" t="inlineStr">
-        <is>
-          <t>Row removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="677">
-      <c r="A677" t="n">
-        <v>285</v>
-      </c>
-      <c r="B677" t="inlineStr">
-        <is>
-          <t>Emp ID</t>
-        </is>
-      </c>
-      <c r="C677" t="inlineStr">
-        <is>
-          <t>EMP1070</t>
-        </is>
-      </c>
-      <c r="D677" t="inlineStr">
-        <is>
-          <t>Duplicate employee ID</t>
-        </is>
-      </c>
-      <c r="E677" t="inlineStr">
-        <is>
-          <t>Row removed</t>
-        </is>
-      </c>
-    </row>
-    <row r="678">
-      <c r="A678" t="n">
-        <v>287</v>
-      </c>
-      <c r="B678" t="inlineStr">
-        <is>
-          <t>Emp ID</t>
-        </is>
-      </c>
-      <c r="C678" t="inlineStr"/>
-      <c r="D678" t="inlineStr">
-        <is>
-          <t>Duplicate employee ID</t>
-        </is>
-      </c>
-      <c r="E678" t="inlineStr">
         <is>
           <t>Row removed</t>
         </is>
@@ -17048,7 +16964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17126,106 +17042,150 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>135</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>EMP1042</t>
-        </is>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mr. Vikram Singh</t>
+          <t>Ajay Reddy</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>176</v>
+        <v>135</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EMP1206</t>
+          <t>EMP1042</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tejaswi Chowdary</t>
+          <t>Mr. Vikram Singh</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EMP1061</t>
+          <t>EMP1206</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rohit Patel</t>
+          <t>Tejaswi Chowdary</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>189</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>EMP1266</t>
-        </is>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Divya Iyer</t>
+          <t>NAVEEN RAO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EMP1179</t>
+          <t>EMP1061</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sneha Chowdary</t>
+          <t>Rohit Patel</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EMP1057</t>
+          <t>EMP1266</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tejaswi Rao</t>
+          <t>Divya Iyer</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>203</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EMP1179</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sneha Chowdary</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>205</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mahesh Khan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>226</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>EMP1057</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Tejaswi Rao</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>268</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>EMP1185</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Rahul Menon</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>287</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pooja Mishra</t>
         </is>
       </c>
     </row>

</xml_diff>